<commit_message>
Intermediate revisions of flouride (F) Template input workbooks.
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Exposure.xlsx
+++ b/Inputs/F_template_parameters_Exposure.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="8_{CCC1AF48-AB15-40A9-B09E-0F30F3DE7B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3F179E8-3192-46FF-B25B-4C9D0660D4BE}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{CCC1AF48-AB15-40A9-B09E-0F30F3DE7B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40F9C257-0C3F-4390-9034-B9A29D1B7DD6}"/>
   <bookViews>
-    <workbookView xWindow="3960" yWindow="810" windowWidth="21825" windowHeight="12915" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="2310" yWindow="0" windowWidth="23325" windowHeight="14670" activeTab="1" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Four_year_old" sheetId="9" r:id="rId1"/>
+    <sheet name="Four_year_old (2)" sheetId="10" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="124">
   <si>
     <t>Code</t>
   </si>
@@ -402,6 +403,9 @@
   </si>
   <si>
     <t>Frac from water:</t>
+  </si>
+  <si>
+    <t>Eight-year-old child</t>
   </si>
 </sst>
 </file>
@@ -489,6 +493,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -789,22 +797,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D6AAA3-4823-45FD-8570-D25DAB8AD8C8}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" customWidth="1"/>
-    <col min="6" max="6" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5859375" customWidth="1"/>
+    <col min="3" max="3" width="15.703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5859375" customWidth="1"/>
+    <col min="5" max="5" width="12.29296875" customWidth="1"/>
+    <col min="6" max="6" width="23.1171875" customWidth="1"/>
+    <col min="7" max="7" width="12.41015625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5859375" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" customWidth="1"/>
-    <col min="12" max="12" width="10.5703125" customWidth="1"/>
+    <col min="10" max="10" width="15.29296875" customWidth="1"/>
+    <col min="12" max="12" width="10.5859375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -824,7 +832,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -838,7 +846,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -849,7 +857,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -860,7 +868,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -877,7 +885,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -894,7 +902,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -908,7 +916,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
@@ -925,7 +933,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>77</v>
       </c>
@@ -939,7 +947,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
@@ -953,7 +961,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -967,7 +975,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -981,7 +989,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
@@ -995,7 +1003,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1012,7 +1020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1027,7 +1035,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1041,7 +1049,7 @@
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
@@ -1058,7 +1066,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -1075,7 +1083,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>85</v>
       </c>
@@ -1095,7 +1103,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1109,7 +1117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1123,7 +1131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1134,7 +1142,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1148,7 +1156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1159,7 +1167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1173,7 +1181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1187,7 +1195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>102</v>
       </c>
@@ -1198,7 +1206,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1229,7 +1237,7 @@
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1266,7 +1274,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
         <v>66</v>
       </c>
@@ -1292,7 +1300,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -1333,7 +1341,7 @@
         <v>0.25680199999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -1354,7 +1362,7 @@
         <v>0.247167889984196</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -1362,7 +1370,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
         <v>98</v>
       </c>
@@ -1373,7 +1381,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>99</v>
       </c>
@@ -1384,7 +1392,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -1395,7 +1403,633 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43F7ED2-4858-4142-B91D-0CDB746679CE}">
+  <dimension ref="A1:M39"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5859375" customWidth="1"/>
+    <col min="3" max="3" width="15.703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5859375" customWidth="1"/>
+    <col min="5" max="5" width="12.29296875" customWidth="1"/>
+    <col min="6" max="6" width="23.1171875" customWidth="1"/>
+    <col min="7" max="7" width="12.41015625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5859375" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="15.29296875" customWidth="1"/>
+    <col min="12" max="12" width="10.5859375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A8" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>251</v>
+      </c>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A17" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17">
+        <v>82.057366080959994</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A18" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18">
+        <v>298</v>
+      </c>
+      <c r="F18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A19" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19">
+        <v>24450</v>
+      </c>
+      <c r="F19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A26" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A28" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A29" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A30" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G30" s="3">
+        <f>40/1000</f>
+        <v>0.04</v>
+      </c>
+      <c r="H30" s="3">
+        <f>21/1000</f>
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="I30" s="3">
+        <f>1.19/1000</f>
+        <v>1.1899999999999999E-3</v>
+      </c>
+      <c r="J30" s="3">
+        <f>0.01/1000</f>
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="K30" s="4">
+        <f>0.442*0.7</f>
+        <v>0.30940000000000001</v>
+      </c>
+      <c r="L30" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A31" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G31" s="3">
+        <v>1</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="J31" s="3">
+        <v>1</v>
+      </c>
+      <c r="K31" s="3">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="A32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3">
+        <f>SUM(G32:K32)/24</f>
+        <v>6.1623000000000004E-2</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G32" s="3">
+        <f>G30*G31*$E$20</f>
+        <v>1</v>
+      </c>
+      <c r="H32" s="3">
+        <f t="shared" ref="H32:J32" si="0">H30*H31*$E$20</f>
+        <v>0.21000000000000002</v>
+      </c>
+      <c r="I32" s="3">
+        <f t="shared" si="0"/>
+        <v>1.1899999999999999E-2</v>
+      </c>
+      <c r="J32" s="3">
+        <f t="shared" si="0"/>
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="K32" s="3">
+        <f t="shared" ref="K32" si="1">K30*K31</f>
+        <v>0.25680199999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A33" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B33" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" t="s">
+        <v>50</v>
+      </c>
+      <c r="F33" t="s">
+        <v>94</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K33" s="5">
+        <f>K32/SUM(G32:K32)</f>
+        <v>0.17363781921252344</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A34" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A35" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A36" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B36" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A37" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -1414,6 +2048,11 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
@@ -1421,12 +2060,52 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1899,52 +2578,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1952,15 +2594,22 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B5A8214-1FA9-425F-8E4E-EB75BD36BC1C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1981,19 +2630,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Parameters in F input files for 4-year-olds updated to match Jean et al. spreadsheet (with calculations included to the side).
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Exposure.xlsx
+++ b/Inputs/F_template_parameters_Exposure.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{CCC1AF48-AB15-40A9-B09E-0F30F3DE7B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40F9C257-0C3F-4390-9034-B9A29D1B7DD6}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="8_{CCC1AF48-AB15-40A9-B09E-0F30F3DE7B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B146AA4-8C1C-476F-A16A-C8D0F0049211}"/>
   <bookViews>
-    <workbookView xWindow="2310" yWindow="0" windowWidth="23325" windowHeight="14670" activeTab="1" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="-25485" yWindow="675" windowWidth="25410" windowHeight="14640" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Four_year_old" sheetId="9" r:id="rId1"/>
-    <sheet name="Four_year_old (2)" sheetId="10" r:id="rId2"/>
+    <sheet name="Eight_year_old" sheetId="10" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="129">
   <si>
     <t>Code</t>
   </si>
@@ -406,12 +406,30 @@
   </si>
   <si>
     <t>Eight-year-old child</t>
+  </si>
+  <si>
+    <t>Net intaked (mg/kg/d)</t>
+  </si>
+  <si>
+    <t>(mg/kg/h)</t>
+  </si>
+  <si>
+    <t>(mg/h)</t>
+  </si>
+  <si>
+    <t>Zero-order infustion</t>
+  </si>
+  <si>
+    <t>Total dose (mg)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -427,7 +445,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -458,6 +476,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -471,13 +495,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -796,23 +822,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D6AAA3-4823-45FD-8570-D25DAB8AD8C8}">
-  <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.5859375" customWidth="1"/>
-    <col min="3" max="3" width="15.703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5859375" customWidth="1"/>
-    <col min="5" max="5" width="12.29296875" customWidth="1"/>
-    <col min="6" max="6" width="23.1171875" customWidth="1"/>
-    <col min="7" max="7" width="12.41015625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5859375" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="15.29296875" customWidth="1"/>
-    <col min="12" max="12" width="10.5859375" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -832,7 +858,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -846,7 +872,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -857,7 +883,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -868,7 +894,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -885,7 +911,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -902,7 +928,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -916,7 +942,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
@@ -933,7 +959,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>77</v>
       </c>
@@ -947,7 +973,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
@@ -961,7 +987,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -975,7 +1001,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -986,10 +1012,10 @@
         <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
@@ -1003,7 +1029,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1020,7 +1046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1031,11 +1057,12 @@
         <v>5</v>
       </c>
       <c r="E16">
-        <v>251</v>
+        <f>2160/24</f>
+        <v>90</v>
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1049,7 +1076,7 @@
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
@@ -1066,7 +1093,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -1083,7 +1110,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>85</v>
       </c>
@@ -1096,14 +1123,14 @@
       <c r="D20">
         <v>0</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="3">
         <v>16</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1117,7 +1144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1130,8 +1157,16 @@
       <c r="D22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="E22" s="3">
+        <f>L32*E23</f>
+        <v>1.9480837499999999</v>
+      </c>
+      <c r="F22">
+        <f>E22*E20</f>
+        <v>31.169339999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1141,8 +1176,11 @@
       <c r="C23" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="E23" s="3">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1156,7 +1194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1167,7 +1205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1181,7 +1219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1195,7 +1233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>102</v>
       </c>
@@ -1206,7 +1244,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1237,7 +1275,7 @@
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1274,7 +1312,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>66</v>
       </c>
@@ -1299,8 +1337,13 @@
       <c r="K31" s="3">
         <v>0.83</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.5">
+      <c r="L31" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -1313,35 +1356,39 @@
       <c r="D32">
         <v>0</v>
       </c>
-      <c r="E32" s="3">
-        <f>SUM(G32:K32)/24</f>
-        <v>4.3290749999999996E-2</v>
-      </c>
       <c r="F32" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G32" s="3">
-        <f>G30*G31*$E$20</f>
-        <v>0.64</v>
+        <f>G30*G31</f>
+        <v>0.04</v>
       </c>
       <c r="H32" s="3">
-        <f t="shared" ref="H32:J32" si="0">H30*H31*$E$20</f>
-        <v>0.13440000000000002</v>
+        <f t="shared" ref="H32:K32" si="0">H30*H31</f>
+        <v>8.4000000000000012E-3</v>
       </c>
       <c r="I32" s="3">
         <f t="shared" si="0"/>
-        <v>7.6159999999999995E-3</v>
+        <v>4.7599999999999997E-4</v>
       </c>
       <c r="J32" s="3">
         <f t="shared" si="0"/>
-        <v>1.6000000000000001E-4</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="K32" s="3">
-        <f t="shared" ref="K32" si="1">K30*K31</f>
-        <v>0.25680199999999997</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
+        <f>K30*K31/E20</f>
+        <v>1.6050124999999998E-2</v>
+      </c>
+      <c r="L32" s="7">
+        <f>SUM($G$32:$K$32)/24</f>
+        <v>2.7056718749999997E-3</v>
+      </c>
+      <c r="M32" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="N32" s="6"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -1351,26 +1398,65 @@
       <c r="C33" t="s">
         <v>50</v>
       </c>
-      <c r="F33" t="s">
-        <v>94</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="K33" s="5">
-        <f>K32/SUM(G32:K32)</f>
-        <v>0.247167889984196</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="F33" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G33" s="3">
+        <f>G32*$E$20</f>
+        <v>0.64</v>
+      </c>
+      <c r="H33" s="3">
+        <f t="shared" ref="H33:K33" si="1">H32*$E$20</f>
+        <v>0.13440000000000002</v>
+      </c>
+      <c r="I33" s="3">
+        <f t="shared" si="1"/>
+        <v>7.6159999999999995E-3</v>
+      </c>
+      <c r="J33" s="3">
+        <f t="shared" si="1"/>
+        <v>1.6000000000000001E-4</v>
+      </c>
+      <c r="K33" s="3">
+        <f t="shared" si="1"/>
+        <v>0.25680199999999997</v>
+      </c>
+      <c r="L33" s="7">
+        <f>SUM($G$33:$K$33)/24</f>
+        <v>4.3290749999999996E-2</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="N33" s="6"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B34" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="F34" t="s">
+        <v>94</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K34" s="5">
+        <f>K33/SUM(G33:K33)</f>
+        <v>0.247167889984196</v>
+      </c>
+      <c r="L34" s="6">
+        <f>L33*E23</f>
+        <v>31.169339999999998</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="N34" s="6"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>98</v>
       </c>
@@ -1381,7 +1467,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>99</v>
       </c>
@@ -1392,7 +1478,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -1403,7 +1489,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -1423,22 +1509,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43F7ED2-4858-4142-B91D-0CDB746679CE}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.5859375" customWidth="1"/>
-    <col min="3" max="3" width="15.703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5859375" customWidth="1"/>
-    <col min="5" max="5" width="12.29296875" customWidth="1"/>
-    <col min="6" max="6" width="23.1171875" customWidth="1"/>
-    <col min="7" max="7" width="12.41015625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5859375" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="15.29296875" customWidth="1"/>
-    <col min="12" max="12" width="10.5859375" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1458,7 +1544,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -1472,7 +1558,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -1483,7 +1569,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -1494,7 +1580,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -1511,7 +1597,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -1528,7 +1614,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -1542,7 +1628,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
@@ -1559,7 +1645,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>77</v>
       </c>
@@ -1573,7 +1659,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
@@ -1587,7 +1673,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -1601,7 +1687,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -1615,7 +1701,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
@@ -1629,7 +1715,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1646,7 +1732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1661,7 +1747,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1675,7 +1761,7 @@
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
@@ -1692,7 +1778,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -1709,7 +1795,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>85</v>
       </c>
@@ -1729,7 +1815,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1743,7 +1829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1757,7 +1843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1768,7 +1854,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1782,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1793,7 +1879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1807,7 +1893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1821,7 +1907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>102</v>
       </c>
@@ -1832,7 +1918,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1863,7 +1949,7 @@
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1900,7 +1986,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>66</v>
       </c>
@@ -1926,7 +2012,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -1967,7 +2053,7 @@
         <v>0.25680199999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -1988,7 +2074,7 @@
         <v>0.17363781921252344</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -1996,7 +2082,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>98</v>
       </c>
@@ -2007,7 +2093,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>99</v>
       </c>
@@ -2018,7 +2104,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -2029,7 +2115,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -2047,65 +2133,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2578,38 +2605,66 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B5A8214-1FA9-425F-8E4E-EB75BD36BC1C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2630,4 +2685,35 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Final tweaks to the model parameter & exposure spreadsheets to provide clear documentation and assure consistency with the published F PBPK model.
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Exposure.xlsx
+++ b/Inputs/F_template_parameters_Exposure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{CCC1AF48-AB15-40A9-B09E-0F30F3DE7B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B146AA4-8C1C-476F-A16A-C8D0F0049211}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="8_{CCC1AF48-AB15-40A9-B09E-0F30F3DE7B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC0C98AC-6E90-442D-B812-E58DCB060E26}"/>
   <bookViews>
-    <workbookView xWindow="-25485" yWindow="675" windowWidth="25410" windowHeight="14640" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView minimized="1" xWindow="-495" yWindow="810" windowWidth="21600" windowHeight="12585" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Four_year_old" sheetId="9" r:id="rId1"/>
@@ -428,7 +428,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -503,7 +503,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -823,22 +823,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D6AAA3-4823-45FD-8570-D25DAB8AD8C8}">
   <dimension ref="A1:N39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" customWidth="1"/>
-    <col min="6" max="6" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.59765625" customWidth="1"/>
+    <col min="3" max="3" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.59765625" customWidth="1"/>
+    <col min="5" max="5" width="12.265625" customWidth="1"/>
+    <col min="6" max="6" width="23.1328125" customWidth="1"/>
+    <col min="7" max="7" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.59765625" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" customWidth="1"/>
-    <col min="12" max="12" width="10.5703125" customWidth="1"/>
+    <col min="10" max="10" width="15.265625" customWidth="1"/>
+    <col min="12" max="12" width="10.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +858,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -872,7 +872,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -883,7 +883,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -894,7 +894,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -911,7 +911,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -928,7 +928,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -942,7 +942,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
@@ -959,7 +959,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>77</v>
       </c>
@@ -973,7 +973,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
@@ -987,7 +987,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -1015,7 +1015,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1076,7 +1076,7 @@
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>85</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>31.169339999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1179,8 +1179,12 @@
       <c r="E23" s="3">
         <v>720</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <f>F22/E23</f>
+        <v>4.3290749999999996E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1194,7 +1198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1205,7 +1209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1219,7 +1223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1233,7 +1237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>102</v>
       </c>
@@ -1244,7 +1248,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1275,7 +1279,7 @@
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1312,7 +1316,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>66</v>
       </c>
@@ -1343,7 +1347,7 @@
       <c r="M31" s="6"/>
       <c r="N31" s="6"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -1364,7 +1368,7 @@
         <v>0.04</v>
       </c>
       <c r="H32" s="3">
-        <f t="shared" ref="H32:K32" si="0">H30*H31</f>
+        <f t="shared" ref="H32:J32" si="0">H30*H31</f>
         <v>8.4000000000000012E-3</v>
       </c>
       <c r="I32" s="3">
@@ -1388,7 +1392,7 @@
       </c>
       <c r="N32" s="6"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -1430,7 +1434,7 @@
       </c>
       <c r="N33" s="6"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -1456,7 +1460,7 @@
       </c>
       <c r="N34" s="6"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>98</v>
       </c>
@@ -1467,7 +1471,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>99</v>
       </c>
@@ -1478,7 +1482,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -1489,7 +1493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -1509,22 +1513,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43F7ED2-4858-4142-B91D-0CDB746679CE}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" customWidth="1"/>
-    <col min="6" max="6" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.59765625" customWidth="1"/>
+    <col min="3" max="3" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.59765625" customWidth="1"/>
+    <col min="5" max="5" width="12.265625" customWidth="1"/>
+    <col min="6" max="6" width="23.1328125" customWidth="1"/>
+    <col min="7" max="7" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.59765625" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" customWidth="1"/>
-    <col min="12" max="12" width="10.5703125" customWidth="1"/>
+    <col min="10" max="10" width="15.265625" customWidth="1"/>
+    <col min="12" max="12" width="10.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1544,7 +1548,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -1558,7 +1562,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -1569,7 +1573,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -1580,7 +1584,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -1597,7 +1601,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -1614,7 +1618,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -1628,7 +1632,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
@@ -1645,7 +1649,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>77</v>
       </c>
@@ -1659,7 +1663,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
@@ -1673,7 +1677,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -1687,7 +1691,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -1701,7 +1705,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
@@ -1715,7 +1719,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1732,7 +1736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1747,7 +1751,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -1761,7 +1765,7 @@
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
@@ -1778,7 +1782,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -1795,7 +1799,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>85</v>
       </c>
@@ -1815,7 +1819,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1829,7 +1833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1843,7 +1847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1854,7 +1858,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1868,7 +1872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1879,7 +1883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1893,7 +1897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1907,7 +1911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>102</v>
       </c>
@@ -1918,7 +1922,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1949,7 +1953,7 @@
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1986,7 +1990,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>66</v>
       </c>
@@ -2012,7 +2016,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -2053,7 +2057,7 @@
         <v>0.25680199999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -2074,7 +2078,7 @@
         <v>0.17363781921252344</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -2082,7 +2086,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>98</v>
       </c>
@@ -2093,7 +2097,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>99</v>
       </c>
@@ -2104,7 +2108,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -2115,7 +2119,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -2133,6 +2137,65 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2605,66 +2668,38 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B5A8214-1FA9-425F-8E4E-EB75BD36BC1C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2685,35 +2720,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>